<commit_message>
args for floor and output stl file
</commit_message>
<xml_diff>
--- a/Greyform-linux-ros1/Greyform-linux-ros1/Python_Application/exporteddatassss(with TMP)(draft)(tetra).xlsx
+++ b/Greyform-linux-ros1/Greyform-linux-ros1/Python_Application/exporteddatassss(with TMP)(draft)(tetra).xlsx
@@ -138,6 +138,289 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -148,11 +431,6 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 0</t>
-        </is>
-      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Marking type</t>
@@ -225,7 +503,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>164</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -247,17 +525,15 @@
       <c r="F2" t="n">
         <v>1.025</v>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G2" t="n">
+        <v>1</v>
       </c>
       <c r="H2" t="n">
         <v>1</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -274,7 +550,7 @@
       <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>167</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -296,17 +572,15 @@
       <c r="F3" t="n">
         <v>0.425</v>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G3" t="n">
+        <v>1</v>
       </c>
       <c r="H3" t="n">
         <v>1</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J3" t="n">
@@ -323,7 +597,7 @@
       <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>165</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -345,17 +619,15 @@
       <c r="F4" t="n">
         <v>-0.775</v>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G4" t="n">
+        <v>1</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J4" t="n">
@@ -372,7 +644,7 @@
       <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
         <v>166</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -394,17 +666,15 @@
       <c r="F5" t="n">
         <v>-0.175</v>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G5" t="n">
+        <v>1</v>
       </c>
       <c r="H5" t="n">
         <v>1</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J5" t="n">
@@ -421,7 +691,7 @@
       <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="1" t="n">
         <v>162</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -443,17 +713,15 @@
       <c r="F6" t="n">
         <v>-0.175</v>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G6" t="n">
+        <v>1</v>
       </c>
       <c r="H6" t="n">
         <v>1</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J6" t="n">
@@ -470,7 +738,7 @@
       <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="1" t="n">
         <v>163</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -492,17 +760,15 @@
       <c r="F7" t="n">
         <v>0.425</v>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G7" t="n">
+        <v>1</v>
       </c>
       <c r="H7" t="n">
         <v>1</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J7" t="n">
@@ -519,7 +785,7 @@
       <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="1" t="n">
         <v>161</v>
       </c>
       <c r="B8" t="inlineStr">
@@ -541,17 +807,15 @@
       <c r="F8" t="n">
         <v>-0.775</v>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G8" t="n">
+        <v>1</v>
       </c>
       <c r="H8" t="n">
         <v>1</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J8" t="n">
@@ -568,7 +832,7 @@
       <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="1" t="n">
         <v>176</v>
       </c>
       <c r="B9" t="inlineStr">
@@ -590,17 +854,15 @@
       <c r="F9" t="n">
         <v>1.025</v>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G9" t="n">
+        <v>1</v>
       </c>
       <c r="H9" t="n">
         <v>1</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J9" t="n">
@@ -617,7 +879,7 @@
       <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="1" t="n">
         <v>175</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -639,17 +901,15 @@
       <c r="F10" t="n">
         <v>0.425</v>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G10" t="n">
+        <v>1</v>
       </c>
       <c r="H10" t="n">
         <v>1</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J10" t="n">
@@ -666,7 +926,7 @@
       <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="1" t="n">
         <v>174</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -688,17 +948,15 @@
       <c r="F11" t="n">
         <v>-0.175</v>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G11" t="n">
+        <v>1</v>
       </c>
       <c r="H11" t="n">
         <v>1</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J11" t="n">
@@ -715,7 +973,7 @@
       <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="1" t="n">
         <v>173</v>
       </c>
       <c r="B12" t="inlineStr">
@@ -737,17 +995,15 @@
       <c r="F12" t="n">
         <v>-0.775</v>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G12" t="n">
+        <v>1</v>
       </c>
       <c r="H12" t="n">
         <v>1</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J12" t="n">
@@ -764,7 +1020,7 @@
       <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="1" t="n">
         <v>172</v>
       </c>
       <c r="B13" t="inlineStr">
@@ -786,17 +1042,15 @@
       <c r="F13" t="n">
         <v>1.025</v>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G13" t="n">
+        <v>1</v>
       </c>
       <c r="H13" t="n">
         <v>1</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J13" t="n">
@@ -813,7 +1067,7 @@
       <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="1" t="n">
         <v>171</v>
       </c>
       <c r="B14" t="inlineStr">
@@ -835,17 +1089,15 @@
       <c r="F14" t="n">
         <v>0.425</v>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G14" t="n">
+        <v>1</v>
       </c>
       <c r="H14" t="n">
         <v>1</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J14" t="n">
@@ -862,7 +1114,7 @@
       <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="1" t="n">
         <v>170</v>
       </c>
       <c r="B15" t="inlineStr">
@@ -884,17 +1136,15 @@
       <c r="F15" t="n">
         <v>-0.175</v>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G15" t="n">
+        <v>1</v>
       </c>
       <c r="H15" t="n">
         <v>1</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J15" t="n">
@@ -911,7 +1161,7 @@
       <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="1" t="n">
         <v>169</v>
       </c>
       <c r="B16" t="inlineStr">
@@ -933,17 +1183,15 @@
       <c r="F16" t="n">
         <v>-0.775</v>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G16" t="n">
+        <v>1</v>
       </c>
       <c r="H16" t="n">
         <v>1</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J16" t="n">
@@ -960,7 +1208,7 @@
       <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="1" t="n">
         <v>168</v>
       </c>
       <c r="B17" t="inlineStr">
@@ -982,17 +1230,15 @@
       <c r="F17" t="n">
         <v>1.025</v>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G17" t="n">
+        <v>1</v>
       </c>
       <c r="H17" t="n">
         <v>1</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J17" t="n">
@@ -1009,7 +1255,7 @@
       <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="1" t="n">
         <v>180</v>
       </c>
       <c r="B18" t="inlineStr">
@@ -1031,17 +1277,15 @@
       <c r="F18" t="n">
         <v>1.025</v>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G18" t="n">
+        <v>1</v>
       </c>
       <c r="H18" t="n">
         <v>1</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J18" t="n">
@@ -1058,7 +1302,7 @@
       <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="1" t="n">
         <v>177</v>
       </c>
       <c r="B19" t="inlineStr">
@@ -1080,17 +1324,15 @@
       <c r="F19" t="n">
         <v>-0.775</v>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G19" t="n">
+        <v>1</v>
       </c>
       <c r="H19" t="n">
         <v>1</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J19" t="n">
@@ -1107,7 +1349,7 @@
       <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="1" t="n">
         <v>178</v>
       </c>
       <c r="B20" t="inlineStr">
@@ -1129,17 +1371,15 @@
       <c r="F20" t="n">
         <v>-0.175</v>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G20" t="n">
+        <v>1</v>
       </c>
       <c r="H20" t="n">
         <v>1</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J20" t="n">
@@ -1156,7 +1396,7 @@
       <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="1" t="n">
         <v>179</v>
       </c>
       <c r="B21" t="inlineStr">
@@ -1178,17 +1418,15 @@
       <c r="F21" t="n">
         <v>0.425</v>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G21" t="n">
+        <v>1</v>
       </c>
       <c r="H21" t="n">
         <v>1</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J21" t="n">
@@ -1205,7 +1443,7 @@
       <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="1" t="n">
         <v>182</v>
       </c>
       <c r="B22" t="inlineStr">
@@ -1227,17 +1465,15 @@
       <c r="F22" t="n">
         <v>-0.175</v>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G22" t="n">
+        <v>1</v>
       </c>
       <c r="H22" t="n">
         <v>1</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J22" t="n">
@@ -1254,7 +1490,7 @@
       <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="1" t="n">
         <v>181</v>
       </c>
       <c r="B23" t="inlineStr">
@@ -1276,17 +1512,15 @@
       <c r="F23" t="n">
         <v>-0.775</v>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G23" t="n">
+        <v>1</v>
       </c>
       <c r="H23" t="n">
         <v>1</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J23" t="n">
@@ -1303,7 +1537,7 @@
       <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" s="1" t="n">
         <v>183</v>
       </c>
       <c r="B24" t="inlineStr">
@@ -1325,17 +1559,15 @@
       <c r="F24" t="n">
         <v>0.425</v>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G24" t="n">
+        <v>1</v>
       </c>
       <c r="H24" t="n">
         <v>1</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J24" t="n">
@@ -1352,7 +1584,7 @@
       <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="n">
+      <c r="A25" s="1" t="n">
         <v>184</v>
       </c>
       <c r="B25" t="inlineStr">
@@ -1374,17 +1606,15 @@
       <c r="F25" t="n">
         <v>1.025</v>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G25" t="n">
+        <v>1</v>
       </c>
       <c r="H25" t="n">
         <v>1</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J25" t="n">
@@ -1401,7 +1631,7 @@
       <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" s="1" t="n">
         <v>187</v>
       </c>
       <c r="B26" t="inlineStr">
@@ -1423,17 +1653,15 @@
       <c r="F26" t="n">
         <v>-0.75</v>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="G26" t="n">
+        <v>2</v>
       </c>
       <c r="H26" t="n">
         <v>1</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J26" t="n">
@@ -1450,7 +1678,7 @@
       <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="n">
+      <c r="A27" s="1" t="n">
         <v>186</v>
       </c>
       <c r="B27" t="inlineStr">
@@ -1472,17 +1700,15 @@
       <c r="F27" t="n">
         <v>-0.15</v>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="G27" t="n">
+        <v>2</v>
       </c>
       <c r="H27" t="n">
         <v>1</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J27" t="n">
@@ -1499,7 +1725,7 @@
       <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="n">
+      <c r="A28" s="1" t="n">
         <v>185</v>
       </c>
       <c r="B28" t="inlineStr">
@@ -1521,17 +1747,15 @@
       <c r="F28" t="n">
         <v>-0.75</v>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="G28" t="n">
+        <v>2</v>
       </c>
       <c r="H28" t="n">
         <v>1</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J28" t="n">
@@ -1548,7 +1772,7 @@
       <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="1" t="n">
         <v>188</v>
       </c>
       <c r="B29" t="inlineStr">
@@ -1570,17 +1794,15 @@
       <c r="F29" t="n">
         <v>-0.15</v>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="G29" t="n">
+        <v>2</v>
       </c>
       <c r="H29" t="n">
         <v>1</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J29" t="n">
@@ -1597,7 +1819,7 @@
       <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="n">
+      <c r="A30" s="1" t="n">
         <v>191</v>
       </c>
       <c r="B30" t="inlineStr">
@@ -1619,17 +1841,15 @@
       <c r="F30" t="n">
         <v>0.425</v>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="G30" t="n">
+        <v>3</v>
       </c>
       <c r="H30" t="n">
         <v>1</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J30" t="n">
@@ -1646,7 +1866,7 @@
       <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="1" t="n">
         <v>190</v>
       </c>
       <c r="B31" t="inlineStr">
@@ -1668,17 +1888,15 @@
       <c r="F31" t="n">
         <v>-0.175</v>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="G31" t="n">
+        <v>3</v>
       </c>
       <c r="H31" t="n">
         <v>1</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J31" t="n">
@@ -1695,7 +1913,7 @@
       <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="n">
+      <c r="A32" s="1" t="n">
         <v>189</v>
       </c>
       <c r="B32" t="inlineStr">
@@ -1717,17 +1935,15 @@
       <c r="F32" t="n">
         <v>-0.775</v>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="G32" t="n">
+        <v>3</v>
       </c>
       <c r="H32" t="n">
         <v>1</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J32" t="n">
@@ -1744,7 +1960,7 @@
       <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="n">
+      <c r="A33" s="1" t="n">
         <v>192</v>
       </c>
       <c r="B33" t="inlineStr">
@@ -1766,17 +1982,15 @@
       <c r="F33" t="n">
         <v>1.025</v>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="G33" t="n">
+        <v>3</v>
       </c>
       <c r="H33" t="n">
         <v>1</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J33" t="n">
@@ -1793,7 +2007,7 @@
       <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="n">
+      <c r="A34" s="1" t="n">
         <v>193</v>
       </c>
       <c r="B34" t="inlineStr">
@@ -1815,17 +2029,15 @@
       <c r="F34" t="n">
         <v>-0.775</v>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="G34" t="n">
+        <v>4</v>
       </c>
       <c r="H34" t="n">
         <v>1</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J34" t="n">
@@ -1842,7 +2054,7 @@
       <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="n">
+      <c r="A35" s="1" t="n">
         <v>194</v>
       </c>
       <c r="B35" t="inlineStr">
@@ -1864,17 +2076,15 @@
       <c r="F35" t="n">
         <v>-0.175</v>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="G35" t="n">
+        <v>4</v>
       </c>
       <c r="H35" t="n">
         <v>1</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J35" t="n">
@@ -1891,7 +2101,7 @@
       <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="n">
+      <c r="A36" s="1" t="n">
         <v>195</v>
       </c>
       <c r="B36" t="inlineStr">
@@ -1913,17 +2123,15 @@
       <c r="F36" t="n">
         <v>0.425</v>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="G36" t="n">
+        <v>4</v>
       </c>
       <c r="H36" t="n">
         <v>1</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J36" t="n">
@@ -1940,7 +2148,7 @@
       <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="n">
+      <c r="A37" s="1" t="n">
         <v>196</v>
       </c>
       <c r="B37" t="inlineStr">
@@ -1962,17 +2170,15 @@
       <c r="F37" t="n">
         <v>1.025</v>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="G37" t="n">
+        <v>4</v>
       </c>
       <c r="H37" t="n">
         <v>1</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J37" t="n">
@@ -1989,7 +2195,7 @@
       <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="n">
+      <c r="A38" s="1" t="n">
         <v>197</v>
       </c>
       <c r="B38" t="inlineStr">
@@ -2011,17 +2217,15 @@
       <c r="F38" t="n">
         <v>-0.775</v>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G38" t="n">
+        <v>5</v>
       </c>
       <c r="H38" t="n">
         <v>1</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J38" t="n">
@@ -2038,7 +2242,7 @@
       <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="1" t="n">
         <v>200</v>
       </c>
       <c r="B39" t="inlineStr">
@@ -2060,17 +2264,15 @@
       <c r="F39" t="n">
         <v>-0.775</v>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G39" t="n">
+        <v>5</v>
       </c>
       <c r="H39" t="n">
         <v>1</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J39" t="n">
@@ -2087,7 +2289,7 @@
       <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="1" t="n">
         <v>201</v>
       </c>
       <c r="B40" t="inlineStr">
@@ -2109,17 +2311,15 @@
       <c r="F40" t="n">
         <v>-0.175</v>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G40" t="n">
+        <v>5</v>
       </c>
       <c r="H40" t="n">
         <v>1</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J40" t="n">
@@ -2136,7 +2336,7 @@
       <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="n">
+      <c r="A41" s="1" t="n">
         <v>202</v>
       </c>
       <c r="B41" t="inlineStr">
@@ -2158,17 +2358,15 @@
       <c r="F41" t="n">
         <v>0.425</v>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G41" t="n">
+        <v>5</v>
       </c>
       <c r="H41" t="n">
         <v>1</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J41" t="n">
@@ -2185,7 +2383,7 @@
       <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" t="n">
+      <c r="A42" s="1" t="n">
         <v>203</v>
       </c>
       <c r="B42" t="inlineStr">
@@ -2207,17 +2405,15 @@
       <c r="F42" t="n">
         <v>1.025</v>
       </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G42" t="n">
+        <v>5</v>
       </c>
       <c r="H42" t="n">
         <v>1</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J42" t="n">
@@ -2234,7 +2430,7 @@
       <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="1" t="n">
         <v>198</v>
       </c>
       <c r="B43" t="inlineStr">
@@ -2256,17 +2452,15 @@
       <c r="F43" t="n">
         <v>-0.775</v>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G43" t="n">
+        <v>5</v>
       </c>
       <c r="H43" t="n">
         <v>1</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J43" t="n">
@@ -2283,7 +2477,7 @@
       <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="n">
+      <c r="A44" s="1" t="n">
         <v>199</v>
       </c>
       <c r="B44" t="inlineStr">
@@ -2305,17 +2499,15 @@
       <c r="F44" t="n">
         <v>-0.775</v>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G44" t="n">
+        <v>5</v>
       </c>
       <c r="H44" t="n">
         <v>1</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J44" t="n">
@@ -2332,7 +2524,7 @@
       <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="1" t="n">
         <v>205</v>
       </c>
       <c r="B45" t="inlineStr">
@@ -2354,17 +2546,15 @@
       <c r="F45" t="n">
         <v>-0.175</v>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="G45" t="n">
+        <v>6</v>
       </c>
       <c r="H45" t="n">
         <v>1</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J45" t="n">
@@ -2381,7 +2571,7 @@
       <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="1" t="n">
         <v>204</v>
       </c>
       <c r="B46" t="inlineStr">
@@ -2403,17 +2593,15 @@
       <c r="F46" t="n">
         <v>-0.775</v>
       </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="G46" t="n">
+        <v>6</v>
       </c>
       <c r="H46" t="n">
         <v>1</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J46" t="n">
@@ -2430,7 +2618,7 @@
       <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" t="n">
+      <c r="A47" s="1" t="n">
         <v>211</v>
       </c>
       <c r="B47" t="inlineStr">
@@ -2452,17 +2640,15 @@
       <c r="F47" t="n">
         <v>1.025</v>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="G47" t="n">
+        <v>6</v>
       </c>
       <c r="H47" t="n">
         <v>1</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J47" t="n">
@@ -2479,7 +2665,7 @@
       <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" t="n">
+      <c r="A48" s="1" t="n">
         <v>210</v>
       </c>
       <c r="B48" t="inlineStr">
@@ -2501,17 +2687,15 @@
       <c r="F48" t="n">
         <v>0.425</v>
       </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="G48" t="n">
+        <v>6</v>
       </c>
       <c r="H48" t="n">
         <v>1</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J48" t="n">
@@ -2528,7 +2712,7 @@
       <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" t="n">
+      <c r="A49" s="1" t="n">
         <v>207</v>
       </c>
       <c r="B49" t="inlineStr">
@@ -2550,17 +2734,15 @@
       <c r="F49" t="n">
         <v>1.025</v>
       </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="G49" t="n">
+        <v>6</v>
       </c>
       <c r="H49" t="n">
         <v>1</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J49" t="n">
@@ -2577,7 +2759,7 @@
       <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" t="n">
+      <c r="A50" s="1" t="n">
         <v>206</v>
       </c>
       <c r="B50" t="inlineStr">
@@ -2599,17 +2781,15 @@
       <c r="F50" t="n">
         <v>0.425</v>
       </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="G50" t="n">
+        <v>6</v>
       </c>
       <c r="H50" t="n">
         <v>1</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J50" t="n">
@@ -2626,7 +2806,7 @@
       <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" t="n">
+      <c r="A51" s="1" t="n">
         <v>209</v>
       </c>
       <c r="B51" t="inlineStr">
@@ -2648,17 +2828,15 @@
       <c r="F51" t="n">
         <v>-0.175</v>
       </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="G51" t="n">
+        <v>6</v>
       </c>
       <c r="H51" t="n">
         <v>1</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J51" t="n">
@@ -2675,7 +2853,7 @@
       <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" t="n">
+      <c r="A52" s="1" t="n">
         <v>208</v>
       </c>
       <c r="B52" t="inlineStr">
@@ -2697,17 +2875,15 @@
       <c r="F52" t="n">
         <v>-0.775</v>
       </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="G52" t="n">
+        <v>6</v>
       </c>
       <c r="H52" t="n">
         <v>1</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J52" t="n">
@@ -2724,7 +2900,7 @@
       <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" t="n">
+      <c r="A53" s="1" t="n">
         <v>215</v>
       </c>
       <c r="B53" t="inlineStr">
@@ -2756,7 +2932,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J53" t="n">
@@ -2773,7 +2949,7 @@
       <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" t="n">
+      <c r="A54" s="1" t="n">
         <v>214</v>
       </c>
       <c r="B54" t="inlineStr">
@@ -2805,7 +2981,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J54" t="n">
@@ -2822,7 +2998,7 @@
       <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" t="n">
+      <c r="A55" s="1" t="n">
         <v>213</v>
       </c>
       <c r="B55" t="inlineStr">
@@ -2854,7 +3030,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J55" t="n">
@@ -2871,7 +3047,7 @@
       <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" t="n">
+      <c r="A56" s="1" t="n">
         <v>212</v>
       </c>
       <c r="B56" t="inlineStr">
@@ -2903,7 +3079,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J56" t="n">
@@ -2920,7 +3096,7 @@
       <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" t="n">
+      <c r="A57" s="1" t="n">
         <v>216</v>
       </c>
       <c r="B57" t="inlineStr">
@@ -2952,7 +3128,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J57" t="n">
@@ -2969,7 +3145,7 @@
       <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" t="n">
+      <c r="A58" s="1" t="n">
         <v>217</v>
       </c>
       <c r="B58" t="inlineStr">
@@ -3001,7 +3177,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J58" t="n">
@@ -3018,7 +3194,7 @@
       <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" t="n">
+      <c r="A59" s="1" t="n">
         <v>218</v>
       </c>
       <c r="B59" t="inlineStr">
@@ -3050,7 +3226,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J59" t="n">
@@ -3067,7 +3243,7 @@
       <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" t="n">
+      <c r="A60" s="1" t="n">
         <v>219</v>
       </c>
       <c r="B60" t="inlineStr">
@@ -3099,7 +3275,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J60" t="n">
@@ -3116,7 +3292,7 @@
       <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" t="n">
+      <c r="A61" s="1" t="n">
         <v>220</v>
       </c>
       <c r="B61" t="inlineStr">
@@ -3148,7 +3324,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J61" t="n">
@@ -3165,7 +3341,7 @@
       <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" t="n">
+      <c r="A62" s="1" t="n">
         <v>221</v>
       </c>
       <c r="B62" t="inlineStr">
@@ -3197,7 +3373,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J62" t="n">
@@ -3214,7 +3390,7 @@
       <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" t="n">
+      <c r="A63" s="1" t="n">
         <v>222</v>
       </c>
       <c r="B63" t="inlineStr">
@@ -3246,7 +3422,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J63" t="n">
@@ -3263,7 +3439,7 @@
       <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" t="n">
+      <c r="A64" s="1" t="n">
         <v>223</v>
       </c>
       <c r="B64" t="inlineStr">
@@ -3295,7 +3471,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J64" t="n">
@@ -3312,7 +3488,7 @@
       <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" t="n">
+      <c r="A65" s="1" t="n">
         <v>224</v>
       </c>
       <c r="B65" t="inlineStr">
@@ -3344,7 +3520,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J65" t="n">
@@ -3361,7 +3537,7 @@
       <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" t="n">
+      <c r="A66" s="1" t="n">
         <v>225</v>
       </c>
       <c r="B66" t="inlineStr">
@@ -3393,7 +3569,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J66" t="n">
@@ -3410,7 +3586,7 @@
       <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" t="n">
+      <c r="A67" s="1" t="n">
         <v>226</v>
       </c>
       <c r="B67" t="inlineStr">
@@ -3442,7 +3618,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J67" t="n">
@@ -3459,7 +3635,7 @@
       <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" t="n">
+      <c r="A68" s="1" t="n">
         <v>227</v>
       </c>
       <c r="B68" t="inlineStr">
@@ -3491,7 +3667,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J68" t="n">
@@ -3508,7 +3684,7 @@
       <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" t="n">
+      <c r="A69" s="1" t="n">
         <v>228</v>
       </c>
       <c r="B69" t="inlineStr">
@@ -3540,7 +3716,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J69" t="n">
@@ -3557,7 +3733,7 @@
       <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" t="n">
+      <c r="A70" s="1" t="n">
         <v>229</v>
       </c>
       <c r="B70" t="inlineStr">
@@ -3589,7 +3765,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J70" t="n">
@@ -3606,7 +3782,7 @@
       <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" t="n">
+      <c r="A71" s="1" t="n">
         <v>230</v>
       </c>
       <c r="B71" t="inlineStr">
@@ -3638,7 +3814,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J71" t="n">
@@ -3655,7 +3831,7 @@
       <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" t="n">
+      <c r="A72" s="1" t="n">
         <v>231</v>
       </c>
       <c r="B72" t="inlineStr">
@@ -3687,7 +3863,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>blank</t>
         </is>
       </c>
       <c r="J72" t="n">
@@ -3718,11 +3894,6 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 0</t>
-        </is>
-      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Marking type</t>
@@ -3795,7 +3966,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>232</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -3817,10 +3988,8 @@
       <c r="F2" t="n">
         <v>0.213</v>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G2" t="n">
+        <v>1</v>
       </c>
       <c r="H2" t="n">
         <v>6</v>
@@ -3844,7 +4013,7 @@
       <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>233</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -3866,10 +4035,8 @@
       <c r="F3" t="n">
         <v>0.213</v>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G3" t="n">
+        <v>1</v>
       </c>
       <c r="H3" t="n">
         <v>6</v>
@@ -3893,7 +4060,7 @@
       <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>234</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -3915,10 +4082,8 @@
       <c r="F4" t="n">
         <v>0.137</v>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G4" t="n">
+        <v>1</v>
       </c>
       <c r="H4" t="n">
         <v>6</v>
@@ -3942,7 +4107,7 @@
       <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
         <v>235</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -3964,10 +4129,8 @@
       <c r="F5" t="n">
         <v>0.137</v>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="G5" t="n">
+        <v>1</v>
       </c>
       <c r="H5" t="n">
         <v>6</v>
@@ -3991,7 +4154,7 @@
       <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="1" t="n">
         <v>236</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -4013,10 +4176,8 @@
       <c r="F6" t="n">
         <v>0.962</v>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="G6" t="n">
+        <v>3</v>
       </c>
       <c r="H6" t="n">
         <v>6</v>
@@ -4040,7 +4201,7 @@
       <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="1" t="n">
         <v>237</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -4062,10 +4223,8 @@
       <c r="F7" t="n">
         <v>0.962</v>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="G7" t="n">
+        <v>3</v>
       </c>
       <c r="H7" t="n">
         <v>6</v>
@@ -4089,7 +4248,7 @@
       <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="1" t="n">
         <v>238</v>
       </c>
       <c r="B8" t="inlineStr">
@@ -4111,10 +4270,8 @@
       <c r="F8" t="n">
         <v>-0.188</v>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="G8" t="n">
+        <v>3</v>
       </c>
       <c r="H8" t="n">
         <v>6</v>
@@ -4138,7 +4295,7 @@
       <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="1" t="n">
         <v>239</v>
       </c>
       <c r="B9" t="inlineStr">
@@ -4160,10 +4317,8 @@
       <c r="F9" t="n">
         <v>-0.188</v>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="G9" t="n">
+        <v>3</v>
       </c>
       <c r="H9" t="n">
         <v>6</v>
@@ -4187,7 +4342,7 @@
       <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="1" t="n">
         <v>240</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -4209,10 +4364,8 @@
       <c r="F10" t="n">
         <v>-0.014</v>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="G10" t="n">
+        <v>3</v>
       </c>
       <c r="H10" t="n">
         <v>6</v>
@@ -4236,7 +4389,7 @@
       <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="1" t="n">
         <v>241</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -4258,10 +4411,8 @@
       <c r="F11" t="n">
         <v>-0.014</v>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="G11" t="n">
+        <v>3</v>
       </c>
       <c r="H11" t="n">
         <v>6</v>
@@ -4285,7 +4436,7 @@
       <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="1" t="n">
         <v>242</v>
       </c>
       <c r="B12" t="inlineStr">
@@ -4307,10 +4458,8 @@
       <c r="F12" t="n">
         <v>-0.08599999999999999</v>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="G12" t="n">
+        <v>3</v>
       </c>
       <c r="H12" t="n">
         <v>6</v>
@@ -4334,7 +4483,7 @@
       <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="1" t="n">
         <v>243</v>
       </c>
       <c r="B13" t="inlineStr">
@@ -4356,10 +4505,8 @@
       <c r="F13" t="n">
         <v>-0.08599999999999999</v>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="G13" t="n">
+        <v>3</v>
       </c>
       <c r="H13" t="n">
         <v>6</v>
@@ -4383,7 +4530,7 @@
       <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="1" t="n">
         <v>5</v>
       </c>
       <c r="B14" t="inlineStr">
@@ -4405,10 +4552,8 @@
       <c r="F14" t="n">
         <v>-0.375</v>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="G14" t="n">
+        <v>4</v>
       </c>
       <c r="H14" t="n">
         <v>6</v>
@@ -4432,7 +4577,7 @@
       <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="1" t="n">
         <v>245</v>
       </c>
       <c r="B15" t="inlineStr">
@@ -4454,10 +4599,8 @@
       <c r="F15" t="n">
         <v>-0.375</v>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="G15" t="n">
+        <v>4</v>
       </c>
       <c r="H15" t="n">
         <v>6</v>
@@ -4481,7 +4624,7 @@
       <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="1" t="n">
         <v>244</v>
       </c>
       <c r="B16" t="inlineStr">
@@ -4503,10 +4646,8 @@
       <c r="F16" t="n">
         <v>-0.375</v>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="G16" t="n">
+        <v>4</v>
       </c>
       <c r="H16" t="n">
         <v>6</v>
@@ -4530,7 +4671,7 @@
       <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="1" t="n">
         <v>247</v>
       </c>
       <c r="B17" t="inlineStr">
@@ -4552,10 +4693,8 @@
       <c r="F17" t="n">
         <v>0.026</v>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G17" t="n">
+        <v>5</v>
       </c>
       <c r="H17" t="n">
         <v>6</v>
@@ -4579,7 +4718,7 @@
       <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="1" t="n">
         <v>246</v>
       </c>
       <c r="B18" t="inlineStr">
@@ -4601,10 +4740,8 @@
       <c r="F18" t="n">
         <v>0.026</v>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G18" t="n">
+        <v>5</v>
       </c>
       <c r="H18" t="n">
         <v>6</v>
@@ -4628,7 +4765,7 @@
       <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="1" t="n">
         <v>92</v>
       </c>
       <c r="B19" t="inlineStr">
@@ -4650,10 +4787,8 @@
       <c r="F19" t="n">
         <v>-0.05</v>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G19" t="n">
+        <v>5</v>
       </c>
       <c r="H19" t="n">
         <v>6</v>
@@ -4677,7 +4812,7 @@
       <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="1" t="n">
         <v>160</v>
       </c>
       <c r="B20" t="inlineStr">
@@ -4699,10 +4834,8 @@
       <c r="F20" t="n">
         <v>0.387</v>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G20" t="n">
+        <v>5</v>
       </c>
       <c r="H20" t="n">
         <v>6</v>
@@ -4726,7 +4859,7 @@
       <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="1" t="n">
         <v>262</v>
       </c>
       <c r="B21" t="inlineStr">
@@ -4748,10 +4881,8 @@
       <c r="F21" t="n">
         <v>-0.75</v>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G21" t="n">
+        <v>5</v>
       </c>
       <c r="H21" t="n">
         <v>6</v>
@@ -4775,7 +4906,7 @@
       <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="1" t="n">
         <v>263</v>
       </c>
       <c r="B22" t="inlineStr">
@@ -4797,10 +4928,8 @@
       <c r="F22" t="n">
         <v>-0.75</v>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G22" t="n">
+        <v>5</v>
       </c>
       <c r="H22" t="n">
         <v>6</v>
@@ -4824,7 +4953,7 @@
       <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="1" t="n">
         <v>255</v>
       </c>
       <c r="B23" t="inlineStr">
@@ -4846,10 +4975,8 @@
       <c r="F23" t="n">
         <v>-0.616</v>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G23" t="n">
+        <v>5</v>
       </c>
       <c r="H23" t="n">
         <v>6</v>
@@ -4873,7 +5000,7 @@
       <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" s="1" t="n">
         <v>254</v>
       </c>
       <c r="B24" t="inlineStr">
@@ -4895,10 +5022,8 @@
       <c r="F24" t="n">
         <v>-0.83</v>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G24" t="n">
+        <v>5</v>
       </c>
       <c r="H24" t="n">
         <v>6</v>
@@ -4922,7 +5047,7 @@
       <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="n">
+      <c r="A25" s="1" t="n">
         <v>261</v>
       </c>
       <c r="B25" t="inlineStr">
@@ -4944,10 +5069,8 @@
       <c r="F25" t="n">
         <v>-0.15</v>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G25" t="n">
+        <v>5</v>
       </c>
       <c r="H25" t="n">
         <v>6</v>
@@ -4971,7 +5094,7 @@
       <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" s="1" t="n">
         <v>260</v>
       </c>
       <c r="B26" t="inlineStr">
@@ -4993,10 +5116,8 @@
       <c r="F26" t="n">
         <v>-0.15</v>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G26" t="n">
+        <v>5</v>
       </c>
       <c r="H26" t="n">
         <v>6</v>
@@ -5020,7 +5141,7 @@
       <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="n">
+      <c r="A27" s="1" t="n">
         <v>259</v>
       </c>
       <c r="B27" t="inlineStr">
@@ -5042,10 +5163,8 @@
       <c r="F27" t="n">
         <v>1.4</v>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G27" t="n">
+        <v>5</v>
       </c>
       <c r="H27" t="n">
         <v>6</v>
@@ -5069,7 +5188,7 @@
       <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="n">
+      <c r="A28" s="1" t="n">
         <v>258</v>
       </c>
       <c r="B28" t="inlineStr">
@@ -5091,10 +5210,8 @@
       <c r="F28" t="n">
         <v>1.4</v>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G28" t="n">
+        <v>5</v>
       </c>
       <c r="H28" t="n">
         <v>6</v>
@@ -5118,7 +5235,7 @@
       <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="1" t="n">
         <v>257</v>
       </c>
       <c r="B29" t="inlineStr">
@@ -5140,10 +5257,8 @@
       <c r="F29" t="n">
         <v>1.4</v>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G29" t="n">
+        <v>5</v>
       </c>
       <c r="H29" t="n">
         <v>6</v>
@@ -5167,7 +5282,7 @@
       <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="n">
+      <c r="A30" s="1" t="n">
         <v>256</v>
       </c>
       <c r="B30" t="inlineStr">
@@ -5189,10 +5304,8 @@
       <c r="F30" t="n">
         <v>1.4</v>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G30" t="n">
+        <v>5</v>
       </c>
       <c r="H30" t="n">
         <v>6</v>
@@ -5216,7 +5329,7 @@
       <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="1" t="n">
         <v>251</v>
       </c>
       <c r="B31" t="inlineStr">
@@ -5238,10 +5351,8 @@
       <c r="F31" t="n">
         <v>-0.402</v>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G31" t="n">
+        <v>5</v>
       </c>
       <c r="H31" t="n">
         <v>6</v>
@@ -5265,7 +5376,7 @@
       <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="n">
+      <c r="A32" s="1" t="n">
         <v>250</v>
       </c>
       <c r="B32" t="inlineStr">
@@ -5287,10 +5398,8 @@
       <c r="F32" t="n">
         <v>-0.22</v>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G32" t="n">
+        <v>5</v>
       </c>
       <c r="H32" t="n">
         <v>6</v>
@@ -5314,7 +5423,7 @@
       <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="n">
+      <c r="A33" s="1" t="n">
         <v>253</v>
       </c>
       <c r="B33" t="inlineStr">
@@ -5336,10 +5445,8 @@
       <c r="F33" t="n">
         <v>-0.83</v>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G33" t="n">
+        <v>5</v>
       </c>
       <c r="H33" t="n">
         <v>6</v>
@@ -5363,7 +5470,7 @@
       <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="n">
+      <c r="A34" s="1" t="n">
         <v>252</v>
       </c>
       <c r="B34" t="inlineStr">
@@ -5385,10 +5492,8 @@
       <c r="F34" t="n">
         <v>-0.402</v>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G34" t="n">
+        <v>5</v>
       </c>
       <c r="H34" t="n">
         <v>6</v>
@@ -5412,7 +5517,7 @@
       <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="n">
+      <c r="A35" s="1" t="n">
         <v>249</v>
       </c>
       <c r="B35" t="inlineStr">
@@ -5434,10 +5539,8 @@
       <c r="F35" t="n">
         <v>-0.466</v>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G35" t="n">
+        <v>5</v>
       </c>
       <c r="H35" t="n">
         <v>6</v>
@@ -5461,7 +5564,7 @@
       <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="n">
+      <c r="A36" s="1" t="n">
         <v>248</v>
       </c>
       <c r="B36" t="inlineStr">
@@ -5483,10 +5586,8 @@
       <c r="F36" t="n">
         <v>-0.466</v>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="G36" t="n">
+        <v>5</v>
       </c>
       <c r="H36" t="n">
         <v>6</v>
@@ -5510,7 +5611,7 @@
       <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="n">
+      <c r="A37" s="1" t="n">
         <v>156</v>
       </c>
       <c r="B37" t="inlineStr">
@@ -5559,7 +5660,7 @@
       <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="n">
+      <c r="A38" s="1" t="n">
         <v>157</v>
       </c>
       <c r="B38" t="inlineStr">
@@ -5608,7 +5709,7 @@
       <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="1" t="n">
         <v>158</v>
       </c>
       <c r="B39" t="inlineStr">
@@ -5657,7 +5758,7 @@
       <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="1" t="n">
         <v>159</v>
       </c>
       <c r="B40" t="inlineStr">
@@ -5706,7 +5807,7 @@
       <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="n">
+      <c r="A41" s="1" t="n">
         <v>4</v>
       </c>
       <c r="B41" t="inlineStr">
@@ -5755,7 +5856,7 @@
       <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" t="n">
+      <c r="A42" s="1" t="n">
         <v>264</v>
       </c>
       <c r="B42" t="inlineStr">
@@ -5804,7 +5905,7 @@
       <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="1" t="n">
         <v>265</v>
       </c>
       <c r="B43" t="inlineStr">
@@ -5853,7 +5954,7 @@
       <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="n">
+      <c r="A44" s="1" t="n">
         <v>266</v>
       </c>
       <c r="B44" t="inlineStr">
@@ -5902,7 +6003,7 @@
       <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="1" t="n">
         <v>267</v>
       </c>
       <c r="B45" t="inlineStr">
@@ -5951,7 +6052,7 @@
       <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="1" t="n">
         <v>268</v>
       </c>
       <c r="B46" t="inlineStr">
@@ -6000,7 +6101,7 @@
       <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" t="n">
+      <c r="A47" s="1" t="n">
         <v>269</v>
       </c>
       <c r="B47" t="inlineStr">
@@ -6049,7 +6150,7 @@
       <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" t="n">
+      <c r="A48" s="1" t="n">
         <v>270</v>
       </c>
       <c r="B48" t="inlineStr">
@@ -6098,7 +6199,7 @@
       <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" t="n">
+      <c r="A49" s="1" t="n">
         <v>271</v>
       </c>
       <c r="B49" t="inlineStr">
@@ -6161,11 +6262,6 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Unnamed: 0</t>
-        </is>
-      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Marking type</t>
@@ -6238,7 +6334,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>20</v>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>